<commit_message>
fix: correct column alignment in review sheets (read his xlsx by header)
His xlsx column order is parameter_name,class,value_type,confidence,
modal_signal,adoc_file,line_number,excerpt - I'd read it positionally and
shifted everything by one (modal_signal column showed the adoc filename).
Rebuilt reading by header name. V3 rows now carry their real modal_signal
(his col 5), adoc_file/line_number in the right columns. Added cell borders
and section shading to params_for_review.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/param_extraction/data/params_for_review.xlsx
+++ b/param_extraction/data/params_for_review.xlsx
@@ -55,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,17 +63,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -448,7 +464,7 @@
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="70" customWidth="1" min="8" max="8"/>
@@ -1127,22 +1143,20 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
+          <t>may cause an illegal-instruction exception or may return a constant value</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
           <t>counters.adoc</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>may cause an illegal-instruction exception or may return a constant value</t>
-        </is>
+      <c r="G16" s="3" t="n">
+        <v>191</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>Accessing an unimplemented counter may cause an illegal-instruction exception or may return a constant value.</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1174,22 +1188,20 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
+          <t>the counter may return a constant value</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
           <t>counters.adoc</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>the counter may return a constant value</t>
-        </is>
+      <c r="G17" s="3" t="n">
+        <v>192</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>If the configuration used to select the events counted by a counter is misconfigured, the counter may return a constant value.</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1221,22 +1233,20 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
+          <t>an implementation may make VSXL be a read-only field</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
           <t>hypervisor.adoc</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>an implementation may make VSXL be a read-only field</t>
-        </is>
+      <c r="G18" s="3" t="n">
+        <v>244</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>In particular, an implementation may make VSXL be a read-only field whose value always ensures that VSXLEN=HSXLEN.</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1268,22 +1278,20 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>An implementation may have WFI always raise a virtual-instruction exception</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
           <t>hypervisor.adoc</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>An implementation may have WFI always raise a virtual-instruction exception</t>
-        </is>
+      <c r="G19" s="3" t="n">
+        <v>260</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>An implementation may have WFI always raise a virtual-instruction exception in VS-mode when VTW=1 (and `mstatus`.TW=0), even if there are pending globally-disabled interrupts when the instruction is executed.</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1315,22 +1323,20 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>An implementation may make field UBE be a read-only copy</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
           <t>hypervisor.adoc</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>An implementation may make field UBE be a read-only copy</t>
-        </is>
+      <c r="G20" s="3" t="n">
+        <v>1226</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>1226</t>
+          <t>An implementation may make field UBE be a read-only copy of `hstatus`.VSBE.</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1362,22 +1368,20 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>An implementation can choose to subset the delegatable traps</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>An implementation can choose to subset the delegatable traps</t>
-        </is>
+      <c r="G21" s="3" t="n">
+        <v>1310</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>1310</t>
+          <t>An implementation can choose to subset the delegatable traps, with the supported delegatable bits found by writing one to every bit location, then reading back the value in `medeleg` or `mideleg` to see which bit positions hold a one.</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1409,22 +1413,20 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
+          <t>may be writable or may be read-only</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>may be writable or may be read-only</t>
-        </is>
+      <c r="G22" s="3" t="n">
+        <v>1395</v>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>1395</t>
+          <t>Each individual bit in register `mip` may be writable or may be read-only.</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1456,22 +1458,20 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
+          <t>Not all physical address bits may be implemented</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
           <t>machine.adoc</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Not all physical address bits may be implemented</t>
-        </is>
+      <c r="G23" s="3" t="n">
+        <v>3395</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>3395</t>
+          <t>Not all physical address bits may be implemented, and so the `pmpaddr` registers are WARL.</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1503,22 +1503,20 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
+          <t>implementations may convert an invalid address</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
           <t>rnmi.adoc</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>implementations may convert an invalid address</t>
-        </is>
+      <c r="G24" s="3" t="n">
+        <v>62</v>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>Prior to writing `mnepc`, implementations may convert an invalid address into some other invalid address that `mnepc` is capable of holding.</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1550,22 +1548,20 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
+          <t>may implement `mseccfg` such that `[s,u]seed` is a read-only constant value</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
           <t>scalar-crypto.adoc</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>may implement `mseccfg` such that `[s,u]seed` is a read-only constant value</t>
-        </is>
+      <c r="G25" s="3" t="n">
+        <v>3750</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>3750</t>
+          <t>Implementations may implement `mseccfg` such that `[s,u]seed` is a read-only constant value `0`.</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -1597,22 +1593,20 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
+          <t>implementation-specific which DEPTH value(s) are supported</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>implementation-specific which DEPTH value(s) are supported</t>
-        </is>
+      <c r="G26" s="3" t="n">
+        <v>189</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>It is implementation-specific which DEPTH value(s) are supported.</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
@@ -1644,22 +1638,20 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
+          <t>The optional MISP bit</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>The optional MISP bit</t>
-        </is>
+      <c r="G27" s="3" t="n">
+        <v>295</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>295</t>
+          <t>The optional MISP bit is set by the hardware when the recorded transfer is an instruction whose target or taken/not-taken direction was mispredicted by the branch predictor. MISP is read-only 0 when not implemented.</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1691,22 +1683,20 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
+          <t>may optionally include a count of CPU cycles</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>may optionally include a count of CPU cycles</t>
-        </is>
+      <c r="G28" s="3" t="n">
+        <v>612</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>612</t>
+          <t>The `ctrdata` register may optionally include a count of CPU cycles elapsed since the prior CTR record.</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1738,22 +1728,20 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
+          <t>may implement 0..4 exponent bits in CCE</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>may implement 0..4 exponent bits in CCE</t>
-        </is>
+      <c r="G29" s="3" t="n">
+        <v>638</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>638</t>
+          <t>An implementation that supports cycle counting must implement CCV and all CCM bits, but may implement 0..4 exponent bits in CCE.</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1785,22 +1773,20 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
+          <t>When the optional `__x__ctrctl`.RASEMU bit is implemented</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
           <t>smctr.adoc</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>When the optional `__x__ctrctl`.RASEMU bit is implemented</t>
-        </is>
+      <c r="G30" s="3" t="n">
+        <v>669</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>669</t>
+          <t>When the optional `__x__ctrctl`.RASEMU bit is implemented and set to 1, transfer recording behavior is altered to emulate the behavior of a return-address stack (RAS).</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -1832,22 +1818,20 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
+          <t>may or may not raise an illegal-instruction or virtual-instruction exception</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
           <t>smstateen.adoc</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>may or may not raise an illegal-instruction or virtual-instruction exception</t>
-        </is>
+      <c r="G31" s="3" t="n">
+        <v>103</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>When a `stateen` CSR prevents access to state for a privilege mode, attempting to execute in that privilege mode an instruction that _implicitly_ updates the state without reading it may or may not raise an illegal-instruction or virtual-instruction exception.</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -1879,22 +1863,20 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
+          <t>an implementation may make UXL be a read-only field</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>an implementation may make UXL be a read-only field</t>
-        </is>
+      <c r="G32" s="3" t="n">
+        <v>134</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>When SXLEN=64, it is a *WARL* field that encodes the current value of UXLEN. In particular, an implementation may make UXL be a read-only field whose value always ensures that UXLEN=SXLEN.</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -1926,22 +1908,20 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
+          <t>it is implementation-defined whether bits SXLEN..XLEN of the destination register are unchanged or are overwritten</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>it is implementation-defined whether bits SXLEN..XLEN of the destination register are unchanged or are overwritten</t>
-        </is>
+      <c r="G33" s="3" t="n">
+        <v>149</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>149</t>
+          <t>When such a HINT is executed with XLEN &lt; SXLEN and bits SXLEN..XLEN of the destination register not all equal to bit XLEN-1, it is implementation-defined whether bits SXLEN..XLEN of the destination register are unchanged or are overwritten with copies of bit XLEN-1.</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -1973,22 +1953,20 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
+          <t>An implementation may make UBE be a read-only field</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>An implementation may make UBE be a read-only field</t>
-        </is>
+      <c r="G34" s="3" t="n">
+        <v>221</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>An implementation may make UBE be a read-only field that always specifies the same endianness as for S-mode.</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2020,22 +1998,20 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
+          <t>may be writable or may be read-only</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>may be writable or may be read-only</t>
-        </is>
+      <c r="G35" s="3" t="n">
+        <v>434</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>Each individual bit in register `sip` may be writable or may be read-only.</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2067,22 +2043,20 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
+          <t>may not be implemented</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>may not be implemented</t>
-        </is>
+      <c r="G36" s="3" t="n">
+        <v>520</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>520</t>
+          <t>Each standard interrupt type (SEI, STI, SSI, or LCOFI) may not be implemented, in which case the corresponding interrupt-pending and interrupt-enable bits are read-only zeros.</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -2114,22 +2088,20 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
+          <t>the implementation may make FIOM read-only zero</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
           <t>supervisor.adoc</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>the implementation may make FIOM read-only zero</t>
-        </is>
+      <c r="G37" s="3" t="n">
+        <v>1001</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>If `satp`.MODE is read-only zero (always Bare), the implementation may make FIOM read-only zero.</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2161,22 +2133,20 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
+          <t>optionally relaxes this alignment requirement</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
           <t>zalasr.adoc</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>optionally relaxes this alignment requirement</t>
-        </is>
+      <c r="G38" s="3" t="n">
+        <v>23</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>The misaligned atomicity granule PMA, defined in Volume II of this manual, optionally relaxes this alignment requirement.</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2208,22 +2178,20 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
+          <t>may define that accesses to certain CSRs are strongly ordered</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
           <t>zicsr.adoc</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>may define that accesses to certain CSRs are strongly ordered</t>
-        </is>
+      <c r="G39" s="3" t="n">
+        <v>244</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>The hardware platform may define that accesses to certain CSRs are strongly ordered, as defined by the Memory-Ordering PMAs section in Volume II of this manual.</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">

</xml_diff>